<commit_message>
Dégustations : date à choisir par téléphone, e-mail ou message (module 1.2.4, Excel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/suivi-degustations.xlsx
+++ b/abc-terroirs/suivi-degustations.xlsx
@@ -16,7 +16,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Achats!$A$1:$M$301</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Reservations!$A$1:$J$301</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">Reservations!$A$1:$K$301</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Seances!$A$1:$I$301</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -95,12 +95,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="60">
   <si>
     <t xml:space="preserve">Suivi des dégustations - ABC Terroirs</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonctionnement : le client achète une ou plusieurs places sur abcterroirs.com, puis appelle le 02 55 54 79 80 pour choisir sa date.</t>
+    <t xml:space="preserve">Fonctionnement : le client achète une ou plusieurs places sur abcterroirs.com, puis choisit sa date par téléphone (02 55 54 79 80), par e-mail (abc3ladmirault@yahoo.com) ou par message.</t>
   </si>
   <si>
     <t xml:space="preserve">1. Achats : à chaque commande de dégustation reçue (mail PrestaShop), ajouter une ligne : date, n° de commande, client, téléphone, dégustation, nombre de places.</t>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">2. Séances : créer une ligne par séance prévue (date, heure, dégustation, boutique). Les places restantes se calculent seules.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Réservations : quand le client appelle, noter son n° de commande, la date et l'heure de la séance, et le nombre de places.</t>
+    <t xml:space="preserve">3. Reservations : quand le client appelle, écrit ou envoie un message, noter son n° de commande, la date et l'heure de la séance, le nombre de places et le moyen utilisé (colonne K).</t>
   </si>
   <si>
     <t xml:space="preserve">   Le nom du client et la dégustation s'affichent automatiquement à partir du n° de commande. Si la séance n'existe pas encore dans « Séances », la colonne « Contrôle » le signale.</t>
@@ -259,7 +259,7 @@
     <t xml:space="preserve">Spi &amp; Bi (Saint-Pierre)</t>
   </si>
   <si>
-    <t xml:space="preserve">Date de l'appel</t>
+    <t xml:space="preserve">Date de la demande</t>
   </si>
   <si>
     <t xml:space="preserve">Date de la séance</t>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t xml:space="preserve">Contrôle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moyen de contact</t>
   </si>
   <si>
     <t xml:space="preserve">Axel</t>
@@ -16307,7 +16310,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J301"/>
+  <dimension ref="A1:K301"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -16320,6 +16323,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16353,6 +16357,9 @@
       <c r="J1" s="3" t="s">
         <v>39</v>
       </c>
+      <c r="K1" s="3" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="n">
@@ -16379,7 +16386,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I2" s="15" t="str">
         <f aca="false">IF(OR(B2="",E2=""),"",IF(COUNTIFS(Seances!$A:$A,E2,Seances!$B:$B,F2,Seances!$C:$C,D2)=0,"Séance à créer dans Seances","OK"))</f>
@@ -16387,6 +16394,9 @@
       </c>
       <c r="J2" s="11" t="s">
         <v>44</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16409,6 +16419,7 @@
         <v/>
       </c>
       <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10"/>
@@ -16430,6 +16441,7 @@
         <v/>
       </c>
       <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10"/>
@@ -16451,6 +16463,7 @@
         <v/>
       </c>
       <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10"/>
@@ -16472,6 +16485,7 @@
         <v/>
       </c>
       <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10"/>
@@ -16493,6 +16507,7 @@
         <v/>
       </c>
       <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10"/>
@@ -16514,6 +16529,7 @@
         <v/>
       </c>
       <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10"/>
@@ -16535,6 +16551,7 @@
         <v/>
       </c>
       <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10"/>
@@ -16556,6 +16573,7 @@
         <v/>
       </c>
       <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10"/>
@@ -16577,6 +16595,7 @@
         <v/>
       </c>
       <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10"/>
@@ -16598,6 +16617,7 @@
         <v/>
       </c>
       <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10"/>
@@ -16619,6 +16639,7 @@
         <v/>
       </c>
       <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10"/>
@@ -16640,6 +16661,7 @@
         <v/>
       </c>
       <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10"/>
@@ -16661,6 +16683,7 @@
         <v/>
       </c>
       <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10"/>
@@ -16682,6 +16705,7 @@
         <v/>
       </c>
       <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10"/>
@@ -16703,6 +16727,7 @@
         <v/>
       </c>
       <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10"/>
@@ -16724,6 +16749,7 @@
         <v/>
       </c>
       <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10"/>
@@ -16745,6 +16771,7 @@
         <v/>
       </c>
       <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10"/>
@@ -16766,6 +16793,7 @@
         <v/>
       </c>
       <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10"/>
@@ -16787,6 +16815,7 @@
         <v/>
       </c>
       <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10"/>
@@ -16808,6 +16837,7 @@
         <v/>
       </c>
       <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10"/>
@@ -16829,6 +16859,7 @@
         <v/>
       </c>
       <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10"/>
@@ -16850,6 +16881,7 @@
         <v/>
       </c>
       <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10"/>
@@ -16871,6 +16903,7 @@
         <v/>
       </c>
       <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10"/>
@@ -16892,6 +16925,7 @@
         <v/>
       </c>
       <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10"/>
@@ -16913,6 +16947,7 @@
         <v/>
       </c>
       <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10"/>
@@ -16934,6 +16969,7 @@
         <v/>
       </c>
       <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10"/>
@@ -16955,6 +16991,7 @@
         <v/>
       </c>
       <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10"/>
@@ -16976,6 +17013,7 @@
         <v/>
       </c>
       <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10"/>
@@ -16997,6 +17035,7 @@
         <v/>
       </c>
       <c r="J31" s="11"/>
+      <c r="K31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10"/>
@@ -17018,6 +17057,7 @@
         <v/>
       </c>
       <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10"/>
@@ -17039,6 +17079,7 @@
         <v/>
       </c>
       <c r="J33" s="11"/>
+      <c r="K33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10"/>
@@ -17060,6 +17101,7 @@
         <v/>
       </c>
       <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10"/>
@@ -17081,6 +17123,7 @@
         <v/>
       </c>
       <c r="J35" s="11"/>
+      <c r="K35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10"/>
@@ -17102,6 +17145,7 @@
         <v/>
       </c>
       <c r="J36" s="11"/>
+      <c r="K36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10"/>
@@ -17123,6 +17167,7 @@
         <v/>
       </c>
       <c r="J37" s="11"/>
+      <c r="K37" s="11"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10"/>
@@ -17144,6 +17189,7 @@
         <v/>
       </c>
       <c r="J38" s="11"/>
+      <c r="K38" s="11"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10"/>
@@ -17165,6 +17211,7 @@
         <v/>
       </c>
       <c r="J39" s="11"/>
+      <c r="K39" s="11"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10"/>
@@ -17186,6 +17233,7 @@
         <v/>
       </c>
       <c r="J40" s="11"/>
+      <c r="K40" s="11"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10"/>
@@ -17207,6 +17255,7 @@
         <v/>
       </c>
       <c r="J41" s="11"/>
+      <c r="K41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10"/>
@@ -17228,6 +17277,7 @@
         <v/>
       </c>
       <c r="J42" s="11"/>
+      <c r="K42" s="11"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10"/>
@@ -17249,6 +17299,7 @@
         <v/>
       </c>
       <c r="J43" s="11"/>
+      <c r="K43" s="11"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10"/>
@@ -17270,6 +17321,7 @@
         <v/>
       </c>
       <c r="J44" s="11"/>
+      <c r="K44" s="11"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10"/>
@@ -17291,6 +17343,7 @@
         <v/>
       </c>
       <c r="J45" s="11"/>
+      <c r="K45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10"/>
@@ -17312,6 +17365,7 @@
         <v/>
       </c>
       <c r="J46" s="11"/>
+      <c r="K46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10"/>
@@ -17333,6 +17387,7 @@
         <v/>
       </c>
       <c r="J47" s="11"/>
+      <c r="K47" s="11"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="10"/>
@@ -17354,6 +17409,7 @@
         <v/>
       </c>
       <c r="J48" s="11"/>
+      <c r="K48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="10"/>
@@ -17375,6 +17431,7 @@
         <v/>
       </c>
       <c r="J49" s="11"/>
+      <c r="K49" s="11"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10"/>
@@ -17396,6 +17453,7 @@
         <v/>
       </c>
       <c r="J50" s="11"/>
+      <c r="K50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10"/>
@@ -17417,6 +17475,7 @@
         <v/>
       </c>
       <c r="J51" s="11"/>
+      <c r="K51" s="11"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="10"/>
@@ -17438,6 +17497,7 @@
         <v/>
       </c>
       <c r="J52" s="11"/>
+      <c r="K52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="10"/>
@@ -17459,6 +17519,7 @@
         <v/>
       </c>
       <c r="J53" s="11"/>
+      <c r="K53" s="11"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10"/>
@@ -17480,6 +17541,7 @@
         <v/>
       </c>
       <c r="J54" s="11"/>
+      <c r="K54" s="11"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10"/>
@@ -17501,6 +17563,7 @@
         <v/>
       </c>
       <c r="J55" s="11"/>
+      <c r="K55" s="11"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="10"/>
@@ -17522,6 +17585,7 @@
         <v/>
       </c>
       <c r="J56" s="11"/>
+      <c r="K56" s="11"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="10"/>
@@ -17543,6 +17607,7 @@
         <v/>
       </c>
       <c r="J57" s="11"/>
+      <c r="K57" s="11"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="10"/>
@@ -17564,6 +17629,7 @@
         <v/>
       </c>
       <c r="J58" s="11"/>
+      <c r="K58" s="11"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="10"/>
@@ -17585,6 +17651,7 @@
         <v/>
       </c>
       <c r="J59" s="11"/>
+      <c r="K59" s="11"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="10"/>
@@ -17606,6 +17673,7 @@
         <v/>
       </c>
       <c r="J60" s="11"/>
+      <c r="K60" s="11"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="10"/>
@@ -17627,6 +17695,7 @@
         <v/>
       </c>
       <c r="J61" s="11"/>
+      <c r="K61" s="11"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10"/>
@@ -17648,6 +17717,7 @@
         <v/>
       </c>
       <c r="J62" s="11"/>
+      <c r="K62" s="11"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="10"/>
@@ -17669,6 +17739,7 @@
         <v/>
       </c>
       <c r="J63" s="11"/>
+      <c r="K63" s="11"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10"/>
@@ -17690,6 +17761,7 @@
         <v/>
       </c>
       <c r="J64" s="11"/>
+      <c r="K64" s="11"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10"/>
@@ -17711,6 +17783,7 @@
         <v/>
       </c>
       <c r="J65" s="11"/>
+      <c r="K65" s="11"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10"/>
@@ -17732,6 +17805,7 @@
         <v/>
       </c>
       <c r="J66" s="11"/>
+      <c r="K66" s="11"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10"/>
@@ -17753,6 +17827,7 @@
         <v/>
       </c>
       <c r="J67" s="11"/>
+      <c r="K67" s="11"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10"/>
@@ -17774,6 +17849,7 @@
         <v/>
       </c>
       <c r="J68" s="11"/>
+      <c r="K68" s="11"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10"/>
@@ -17795,6 +17871,7 @@
         <v/>
       </c>
       <c r="J69" s="11"/>
+      <c r="K69" s="11"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="10"/>
@@ -17816,6 +17893,7 @@
         <v/>
       </c>
       <c r="J70" s="11"/>
+      <c r="K70" s="11"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="10"/>
@@ -17837,6 +17915,7 @@
         <v/>
       </c>
       <c r="J71" s="11"/>
+      <c r="K71" s="11"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10"/>
@@ -17858,6 +17937,7 @@
         <v/>
       </c>
       <c r="J72" s="11"/>
+      <c r="K72" s="11"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10"/>
@@ -17879,6 +17959,7 @@
         <v/>
       </c>
       <c r="J73" s="11"/>
+      <c r="K73" s="11"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="10"/>
@@ -17900,6 +17981,7 @@
         <v/>
       </c>
       <c r="J74" s="11"/>
+      <c r="K74" s="11"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="10"/>
@@ -17921,6 +18003,7 @@
         <v/>
       </c>
       <c r="J75" s="11"/>
+      <c r="K75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="10"/>
@@ -17942,6 +18025,7 @@
         <v/>
       </c>
       <c r="J76" s="11"/>
+      <c r="K76" s="11"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="10"/>
@@ -17963,6 +18047,7 @@
         <v/>
       </c>
       <c r="J77" s="11"/>
+      <c r="K77" s="11"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="10"/>
@@ -17984,6 +18069,7 @@
         <v/>
       </c>
       <c r="J78" s="11"/>
+      <c r="K78" s="11"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="10"/>
@@ -18005,6 +18091,7 @@
         <v/>
       </c>
       <c r="J79" s="11"/>
+      <c r="K79" s="11"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="10"/>
@@ -18026,6 +18113,7 @@
         <v/>
       </c>
       <c r="J80" s="11"/>
+      <c r="K80" s="11"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="10"/>
@@ -18047,6 +18135,7 @@
         <v/>
       </c>
       <c r="J81" s="11"/>
+      <c r="K81" s="11"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="10"/>
@@ -18068,6 +18157,7 @@
         <v/>
       </c>
       <c r="J82" s="11"/>
+      <c r="K82" s="11"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="10"/>
@@ -18089,6 +18179,7 @@
         <v/>
       </c>
       <c r="J83" s="11"/>
+      <c r="K83" s="11"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="10"/>
@@ -18110,6 +18201,7 @@
         <v/>
       </c>
       <c r="J84" s="11"/>
+      <c r="K84" s="11"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="10"/>
@@ -18131,6 +18223,7 @@
         <v/>
       </c>
       <c r="J85" s="11"/>
+      <c r="K85" s="11"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="10"/>
@@ -18152,6 +18245,7 @@
         <v/>
       </c>
       <c r="J86" s="11"/>
+      <c r="K86" s="11"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="10"/>
@@ -18173,6 +18267,7 @@
         <v/>
       </c>
       <c r="J87" s="11"/>
+      <c r="K87" s="11"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="10"/>
@@ -18194,6 +18289,7 @@
         <v/>
       </c>
       <c r="J88" s="11"/>
+      <c r="K88" s="11"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="10"/>
@@ -18215,6 +18311,7 @@
         <v/>
       </c>
       <c r="J89" s="11"/>
+      <c r="K89" s="11"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="10"/>
@@ -18236,6 +18333,7 @@
         <v/>
       </c>
       <c r="J90" s="11"/>
+      <c r="K90" s="11"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="10"/>
@@ -18257,6 +18355,7 @@
         <v/>
       </c>
       <c r="J91" s="11"/>
+      <c r="K91" s="11"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="10"/>
@@ -18278,6 +18377,7 @@
         <v/>
       </c>
       <c r="J92" s="11"/>
+      <c r="K92" s="11"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="10"/>
@@ -18299,6 +18399,7 @@
         <v/>
       </c>
       <c r="J93" s="11"/>
+      <c r="K93" s="11"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="10"/>
@@ -18320,6 +18421,7 @@
         <v/>
       </c>
       <c r="J94" s="11"/>
+      <c r="K94" s="11"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="10"/>
@@ -18341,6 +18443,7 @@
         <v/>
       </c>
       <c r="J95" s="11"/>
+      <c r="K95" s="11"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="10"/>
@@ -18362,6 +18465,7 @@
         <v/>
       </c>
       <c r="J96" s="11"/>
+      <c r="K96" s="11"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="10"/>
@@ -18383,6 +18487,7 @@
         <v/>
       </c>
       <c r="J97" s="11"/>
+      <c r="K97" s="11"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="10"/>
@@ -18404,6 +18509,7 @@
         <v/>
       </c>
       <c r="J98" s="11"/>
+      <c r="K98" s="11"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="10"/>
@@ -18425,6 +18531,7 @@
         <v/>
       </c>
       <c r="J99" s="11"/>
+      <c r="K99" s="11"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="10"/>
@@ -18446,6 +18553,7 @@
         <v/>
       </c>
       <c r="J100" s="11"/>
+      <c r="K100" s="11"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="10"/>
@@ -18467,6 +18575,7 @@
         <v/>
       </c>
       <c r="J101" s="11"/>
+      <c r="K101" s="11"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="10"/>
@@ -18488,6 +18597,7 @@
         <v/>
       </c>
       <c r="J102" s="11"/>
+      <c r="K102" s="11"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="10"/>
@@ -18509,6 +18619,7 @@
         <v/>
       </c>
       <c r="J103" s="11"/>
+      <c r="K103" s="11"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="10"/>
@@ -18530,6 +18641,7 @@
         <v/>
       </c>
       <c r="J104" s="11"/>
+      <c r="K104" s="11"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="10"/>
@@ -18551,6 +18663,7 @@
         <v/>
       </c>
       <c r="J105" s="11"/>
+      <c r="K105" s="11"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="10"/>
@@ -18572,6 +18685,7 @@
         <v/>
       </c>
       <c r="J106" s="11"/>
+      <c r="K106" s="11"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="10"/>
@@ -18593,6 +18707,7 @@
         <v/>
       </c>
       <c r="J107" s="11"/>
+      <c r="K107" s="11"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="10"/>
@@ -18614,6 +18729,7 @@
         <v/>
       </c>
       <c r="J108" s="11"/>
+      <c r="K108" s="11"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="10"/>
@@ -18635,6 +18751,7 @@
         <v/>
       </c>
       <c r="J109" s="11"/>
+      <c r="K109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="10"/>
@@ -18656,6 +18773,7 @@
         <v/>
       </c>
       <c r="J110" s="11"/>
+      <c r="K110" s="11"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="10"/>
@@ -18677,6 +18795,7 @@
         <v/>
       </c>
       <c r="J111" s="11"/>
+      <c r="K111" s="11"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="10"/>
@@ -18698,6 +18817,7 @@
         <v/>
       </c>
       <c r="J112" s="11"/>
+      <c r="K112" s="11"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="10"/>
@@ -18719,6 +18839,7 @@
         <v/>
       </c>
       <c r="J113" s="11"/>
+      <c r="K113" s="11"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="10"/>
@@ -18740,6 +18861,7 @@
         <v/>
       </c>
       <c r="J114" s="11"/>
+      <c r="K114" s="11"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="10"/>
@@ -18761,6 +18883,7 @@
         <v/>
       </c>
       <c r="J115" s="11"/>
+      <c r="K115" s="11"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="10"/>
@@ -18782,6 +18905,7 @@
         <v/>
       </c>
       <c r="J116" s="11"/>
+      <c r="K116" s="11"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="10"/>
@@ -18803,6 +18927,7 @@
         <v/>
       </c>
       <c r="J117" s="11"/>
+      <c r="K117" s="11"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="10"/>
@@ -18824,6 +18949,7 @@
         <v/>
       </c>
       <c r="J118" s="11"/>
+      <c r="K118" s="11"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="10"/>
@@ -18845,6 +18971,7 @@
         <v/>
       </c>
       <c r="J119" s="11"/>
+      <c r="K119" s="11"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="10"/>
@@ -18866,6 +18993,7 @@
         <v/>
       </c>
       <c r="J120" s="11"/>
+      <c r="K120" s="11"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="10"/>
@@ -18887,6 +19015,7 @@
         <v/>
       </c>
       <c r="J121" s="11"/>
+      <c r="K121" s="11"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="10"/>
@@ -18908,6 +19037,7 @@
         <v/>
       </c>
       <c r="J122" s="11"/>
+      <c r="K122" s="11"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="10"/>
@@ -18929,6 +19059,7 @@
         <v/>
       </c>
       <c r="J123" s="11"/>
+      <c r="K123" s="11"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="10"/>
@@ -18950,6 +19081,7 @@
         <v/>
       </c>
       <c r="J124" s="11"/>
+      <c r="K124" s="11"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="10"/>
@@ -18971,6 +19103,7 @@
         <v/>
       </c>
       <c r="J125" s="11"/>
+      <c r="K125" s="11"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="10"/>
@@ -18992,6 +19125,7 @@
         <v/>
       </c>
       <c r="J126" s="11"/>
+      <c r="K126" s="11"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="10"/>
@@ -19013,6 +19147,7 @@
         <v/>
       </c>
       <c r="J127" s="11"/>
+      <c r="K127" s="11"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="10"/>
@@ -19034,6 +19169,7 @@
         <v/>
       </c>
       <c r="J128" s="11"/>
+      <c r="K128" s="11"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="10"/>
@@ -19055,6 +19191,7 @@
         <v/>
       </c>
       <c r="J129" s="11"/>
+      <c r="K129" s="11"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="10"/>
@@ -19076,6 +19213,7 @@
         <v/>
       </c>
       <c r="J130" s="11"/>
+      <c r="K130" s="11"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="10"/>
@@ -19097,6 +19235,7 @@
         <v/>
       </c>
       <c r="J131" s="11"/>
+      <c r="K131" s="11"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="10"/>
@@ -19118,6 +19257,7 @@
         <v/>
       </c>
       <c r="J132" s="11"/>
+      <c r="K132" s="11"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="10"/>
@@ -19139,6 +19279,7 @@
         <v/>
       </c>
       <c r="J133" s="11"/>
+      <c r="K133" s="11"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="10"/>
@@ -19160,6 +19301,7 @@
         <v/>
       </c>
       <c r="J134" s="11"/>
+      <c r="K134" s="11"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="10"/>
@@ -19181,6 +19323,7 @@
         <v/>
       </c>
       <c r="J135" s="11"/>
+      <c r="K135" s="11"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="10"/>
@@ -19202,6 +19345,7 @@
         <v/>
       </c>
       <c r="J136" s="11"/>
+      <c r="K136" s="11"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="10"/>
@@ -19223,6 +19367,7 @@
         <v/>
       </c>
       <c r="J137" s="11"/>
+      <c r="K137" s="11"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="10"/>
@@ -19244,6 +19389,7 @@
         <v/>
       </c>
       <c r="J138" s="11"/>
+      <c r="K138" s="11"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="10"/>
@@ -19265,6 +19411,7 @@
         <v/>
       </c>
       <c r="J139" s="11"/>
+      <c r="K139" s="11"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="10"/>
@@ -19286,6 +19433,7 @@
         <v/>
       </c>
       <c r="J140" s="11"/>
+      <c r="K140" s="11"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="10"/>
@@ -19307,6 +19455,7 @@
         <v/>
       </c>
       <c r="J141" s="11"/>
+      <c r="K141" s="11"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="10"/>
@@ -19328,6 +19477,7 @@
         <v/>
       </c>
       <c r="J142" s="11"/>
+      <c r="K142" s="11"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="10"/>
@@ -19349,6 +19499,7 @@
         <v/>
       </c>
       <c r="J143" s="11"/>
+      <c r="K143" s="11"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="10"/>
@@ -19370,6 +19521,7 @@
         <v/>
       </c>
       <c r="J144" s="11"/>
+      <c r="K144" s="11"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="10"/>
@@ -19391,6 +19543,7 @@
         <v/>
       </c>
       <c r="J145" s="11"/>
+      <c r="K145" s="11"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="10"/>
@@ -19412,6 +19565,7 @@
         <v/>
       </c>
       <c r="J146" s="11"/>
+      <c r="K146" s="11"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="10"/>
@@ -19433,6 +19587,7 @@
         <v/>
       </c>
       <c r="J147" s="11"/>
+      <c r="K147" s="11"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="10"/>
@@ -19454,6 +19609,7 @@
         <v/>
       </c>
       <c r="J148" s="11"/>
+      <c r="K148" s="11"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="10"/>
@@ -19475,6 +19631,7 @@
         <v/>
       </c>
       <c r="J149" s="11"/>
+      <c r="K149" s="11"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="10"/>
@@ -19496,6 +19653,7 @@
         <v/>
       </c>
       <c r="J150" s="11"/>
+      <c r="K150" s="11"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="10"/>
@@ -19517,6 +19675,7 @@
         <v/>
       </c>
       <c r="J151" s="11"/>
+      <c r="K151" s="11"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="10"/>
@@ -19538,6 +19697,7 @@
         <v/>
       </c>
       <c r="J152" s="11"/>
+      <c r="K152" s="11"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="10"/>
@@ -19559,6 +19719,7 @@
         <v/>
       </c>
       <c r="J153" s="11"/>
+      <c r="K153" s="11"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="10"/>
@@ -19580,6 +19741,7 @@
         <v/>
       </c>
       <c r="J154" s="11"/>
+      <c r="K154" s="11"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="10"/>
@@ -19601,6 +19763,7 @@
         <v/>
       </c>
       <c r="J155" s="11"/>
+      <c r="K155" s="11"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="10"/>
@@ -19622,6 +19785,7 @@
         <v/>
       </c>
       <c r="J156" s="11"/>
+      <c r="K156" s="11"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="10"/>
@@ -19643,6 +19807,7 @@
         <v/>
       </c>
       <c r="J157" s="11"/>
+      <c r="K157" s="11"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="10"/>
@@ -19664,6 +19829,7 @@
         <v/>
       </c>
       <c r="J158" s="11"/>
+      <c r="K158" s="11"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="10"/>
@@ -19685,6 +19851,7 @@
         <v/>
       </c>
       <c r="J159" s="11"/>
+      <c r="K159" s="11"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="10"/>
@@ -19706,6 +19873,7 @@
         <v/>
       </c>
       <c r="J160" s="11"/>
+      <c r="K160" s="11"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="10"/>
@@ -19727,6 +19895,7 @@
         <v/>
       </c>
       <c r="J161" s="11"/>
+      <c r="K161" s="11"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="10"/>
@@ -19748,6 +19917,7 @@
         <v/>
       </c>
       <c r="J162" s="11"/>
+      <c r="K162" s="11"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="10"/>
@@ -19769,6 +19939,7 @@
         <v/>
       </c>
       <c r="J163" s="11"/>
+      <c r="K163" s="11"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="10"/>
@@ -19790,6 +19961,7 @@
         <v/>
       </c>
       <c r="J164" s="11"/>
+      <c r="K164" s="11"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="10"/>
@@ -19811,6 +19983,7 @@
         <v/>
       </c>
       <c r="J165" s="11"/>
+      <c r="K165" s="11"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="10"/>
@@ -19832,6 +20005,7 @@
         <v/>
       </c>
       <c r="J166" s="11"/>
+      <c r="K166" s="11"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="10"/>
@@ -19853,6 +20027,7 @@
         <v/>
       </c>
       <c r="J167" s="11"/>
+      <c r="K167" s="11"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="10"/>
@@ -19874,6 +20049,7 @@
         <v/>
       </c>
       <c r="J168" s="11"/>
+      <c r="K168" s="11"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="10"/>
@@ -19895,6 +20071,7 @@
         <v/>
       </c>
       <c r="J169" s="11"/>
+      <c r="K169" s="11"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="10"/>
@@ -19916,6 +20093,7 @@
         <v/>
       </c>
       <c r="J170" s="11"/>
+      <c r="K170" s="11"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="10"/>
@@ -19937,6 +20115,7 @@
         <v/>
       </c>
       <c r="J171" s="11"/>
+      <c r="K171" s="11"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="10"/>
@@ -19958,6 +20137,7 @@
         <v/>
       </c>
       <c r="J172" s="11"/>
+      <c r="K172" s="11"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="10"/>
@@ -19979,6 +20159,7 @@
         <v/>
       </c>
       <c r="J173" s="11"/>
+      <c r="K173" s="11"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="10"/>
@@ -20000,6 +20181,7 @@
         <v/>
       </c>
       <c r="J174" s="11"/>
+      <c r="K174" s="11"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="10"/>
@@ -20021,6 +20203,7 @@
         <v/>
       </c>
       <c r="J175" s="11"/>
+      <c r="K175" s="11"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="10"/>
@@ -20042,6 +20225,7 @@
         <v/>
       </c>
       <c r="J176" s="11"/>
+      <c r="K176" s="11"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="10"/>
@@ -20063,6 +20247,7 @@
         <v/>
       </c>
       <c r="J177" s="11"/>
+      <c r="K177" s="11"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="10"/>
@@ -20084,6 +20269,7 @@
         <v/>
       </c>
       <c r="J178" s="11"/>
+      <c r="K178" s="11"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="10"/>
@@ -20105,6 +20291,7 @@
         <v/>
       </c>
       <c r="J179" s="11"/>
+      <c r="K179" s="11"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="10"/>
@@ -20126,6 +20313,7 @@
         <v/>
       </c>
       <c r="J180" s="11"/>
+      <c r="K180" s="11"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="10"/>
@@ -20147,6 +20335,7 @@
         <v/>
       </c>
       <c r="J181" s="11"/>
+      <c r="K181" s="11"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="10"/>
@@ -20168,6 +20357,7 @@
         <v/>
       </c>
       <c r="J182" s="11"/>
+      <c r="K182" s="11"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="10"/>
@@ -20189,6 +20379,7 @@
         <v/>
       </c>
       <c r="J183" s="11"/>
+      <c r="K183" s="11"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="10"/>
@@ -20210,6 +20401,7 @@
         <v/>
       </c>
       <c r="J184" s="11"/>
+      <c r="K184" s="11"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="10"/>
@@ -20231,6 +20423,7 @@
         <v/>
       </c>
       <c r="J185" s="11"/>
+      <c r="K185" s="11"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="10"/>
@@ -20252,6 +20445,7 @@
         <v/>
       </c>
       <c r="J186" s="11"/>
+      <c r="K186" s="11"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="10"/>
@@ -20273,6 +20467,7 @@
         <v/>
       </c>
       <c r="J187" s="11"/>
+      <c r="K187" s="11"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="10"/>
@@ -20294,6 +20489,7 @@
         <v/>
       </c>
       <c r="J188" s="11"/>
+      <c r="K188" s="11"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="10"/>
@@ -20315,6 +20511,7 @@
         <v/>
       </c>
       <c r="J189" s="11"/>
+      <c r="K189" s="11"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="10"/>
@@ -20336,6 +20533,7 @@
         <v/>
       </c>
       <c r="J190" s="11"/>
+      <c r="K190" s="11"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="10"/>
@@ -20357,6 +20555,7 @@
         <v/>
       </c>
       <c r="J191" s="11"/>
+      <c r="K191" s="11"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="10"/>
@@ -20378,6 +20577,7 @@
         <v/>
       </c>
       <c r="J192" s="11"/>
+      <c r="K192" s="11"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="10"/>
@@ -20399,6 +20599,7 @@
         <v/>
       </c>
       <c r="J193" s="11"/>
+      <c r="K193" s="11"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="10"/>
@@ -20420,6 +20621,7 @@
         <v/>
       </c>
       <c r="J194" s="11"/>
+      <c r="K194" s="11"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="10"/>
@@ -20441,6 +20643,7 @@
         <v/>
       </c>
       <c r="J195" s="11"/>
+      <c r="K195" s="11"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="10"/>
@@ -20462,6 +20665,7 @@
         <v/>
       </c>
       <c r="J196" s="11"/>
+      <c r="K196" s="11"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="10"/>
@@ -20483,6 +20687,7 @@
         <v/>
       </c>
       <c r="J197" s="11"/>
+      <c r="K197" s="11"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="10"/>
@@ -20504,6 +20709,7 @@
         <v/>
       </c>
       <c r="J198" s="11"/>
+      <c r="K198" s="11"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="10"/>
@@ -20525,6 +20731,7 @@
         <v/>
       </c>
       <c r="J199" s="11"/>
+      <c r="K199" s="11"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="10"/>
@@ -20546,6 +20753,7 @@
         <v/>
       </c>
       <c r="J200" s="11"/>
+      <c r="K200" s="11"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="10"/>
@@ -20567,6 +20775,7 @@
         <v/>
       </c>
       <c r="J201" s="11"/>
+      <c r="K201" s="11"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="10"/>
@@ -20588,6 +20797,7 @@
         <v/>
       </c>
       <c r="J202" s="11"/>
+      <c r="K202" s="11"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="10"/>
@@ -20609,6 +20819,7 @@
         <v/>
       </c>
       <c r="J203" s="11"/>
+      <c r="K203" s="11"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="10"/>
@@ -20630,6 +20841,7 @@
         <v/>
       </c>
       <c r="J204" s="11"/>
+      <c r="K204" s="11"/>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="10"/>
@@ -20651,6 +20863,7 @@
         <v/>
       </c>
       <c r="J205" s="11"/>
+      <c r="K205" s="11"/>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A206" s="10"/>
@@ -20672,6 +20885,7 @@
         <v/>
       </c>
       <c r="J206" s="11"/>
+      <c r="K206" s="11"/>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="10"/>
@@ -20693,6 +20907,7 @@
         <v/>
       </c>
       <c r="J207" s="11"/>
+      <c r="K207" s="11"/>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="10"/>
@@ -20714,6 +20929,7 @@
         <v/>
       </c>
       <c r="J208" s="11"/>
+      <c r="K208" s="11"/>
     </row>
     <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="10"/>
@@ -20735,6 +20951,7 @@
         <v/>
       </c>
       <c r="J209" s="11"/>
+      <c r="K209" s="11"/>
     </row>
     <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="10"/>
@@ -20756,6 +20973,7 @@
         <v/>
       </c>
       <c r="J210" s="11"/>
+      <c r="K210" s="11"/>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="10"/>
@@ -20777,6 +20995,7 @@
         <v/>
       </c>
       <c r="J211" s="11"/>
+      <c r="K211" s="11"/>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="10"/>
@@ -20798,6 +21017,7 @@
         <v/>
       </c>
       <c r="J212" s="11"/>
+      <c r="K212" s="11"/>
     </row>
     <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="10"/>
@@ -20819,6 +21039,7 @@
         <v/>
       </c>
       <c r="J213" s="11"/>
+      <c r="K213" s="11"/>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="10"/>
@@ -20840,6 +21061,7 @@
         <v/>
       </c>
       <c r="J214" s="11"/>
+      <c r="K214" s="11"/>
     </row>
     <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="10"/>
@@ -20861,6 +21083,7 @@
         <v/>
       </c>
       <c r="J215" s="11"/>
+      <c r="K215" s="11"/>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="10"/>
@@ -20882,6 +21105,7 @@
         <v/>
       </c>
       <c r="J216" s="11"/>
+      <c r="K216" s="11"/>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="10"/>
@@ -20903,6 +21127,7 @@
         <v/>
       </c>
       <c r="J217" s="11"/>
+      <c r="K217" s="11"/>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="10"/>
@@ -20924,6 +21149,7 @@
         <v/>
       </c>
       <c r="J218" s="11"/>
+      <c r="K218" s="11"/>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="10"/>
@@ -20945,6 +21171,7 @@
         <v/>
       </c>
       <c r="J219" s="11"/>
+      <c r="K219" s="11"/>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="10"/>
@@ -20966,6 +21193,7 @@
         <v/>
       </c>
       <c r="J220" s="11"/>
+      <c r="K220" s="11"/>
     </row>
     <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="10"/>
@@ -20987,6 +21215,7 @@
         <v/>
       </c>
       <c r="J221" s="11"/>
+      <c r="K221" s="11"/>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="10"/>
@@ -21008,6 +21237,7 @@
         <v/>
       </c>
       <c r="J222" s="11"/>
+      <c r="K222" s="11"/>
     </row>
     <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="10"/>
@@ -21029,6 +21259,7 @@
         <v/>
       </c>
       <c r="J223" s="11"/>
+      <c r="K223" s="11"/>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="10"/>
@@ -21050,6 +21281,7 @@
         <v/>
       </c>
       <c r="J224" s="11"/>
+      <c r="K224" s="11"/>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="10"/>
@@ -21071,6 +21303,7 @@
         <v/>
       </c>
       <c r="J225" s="11"/>
+      <c r="K225" s="11"/>
     </row>
     <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="10"/>
@@ -21092,6 +21325,7 @@
         <v/>
       </c>
       <c r="J226" s="11"/>
+      <c r="K226" s="11"/>
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="10"/>
@@ -21113,6 +21347,7 @@
         <v/>
       </c>
       <c r="J227" s="11"/>
+      <c r="K227" s="11"/>
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="10"/>
@@ -21134,6 +21369,7 @@
         <v/>
       </c>
       <c r="J228" s="11"/>
+      <c r="K228" s="11"/>
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="10"/>
@@ -21155,6 +21391,7 @@
         <v/>
       </c>
       <c r="J229" s="11"/>
+      <c r="K229" s="11"/>
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="10"/>
@@ -21176,6 +21413,7 @@
         <v/>
       </c>
       <c r="J230" s="11"/>
+      <c r="K230" s="11"/>
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="10"/>
@@ -21197,6 +21435,7 @@
         <v/>
       </c>
       <c r="J231" s="11"/>
+      <c r="K231" s="11"/>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="10"/>
@@ -21218,6 +21457,7 @@
         <v/>
       </c>
       <c r="J232" s="11"/>
+      <c r="K232" s="11"/>
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="10"/>
@@ -21239,6 +21479,7 @@
         <v/>
       </c>
       <c r="J233" s="11"/>
+      <c r="K233" s="11"/>
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="10"/>
@@ -21260,6 +21501,7 @@
         <v/>
       </c>
       <c r="J234" s="11"/>
+      <c r="K234" s="11"/>
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="10"/>
@@ -21281,6 +21523,7 @@
         <v/>
       </c>
       <c r="J235" s="11"/>
+      <c r="K235" s="11"/>
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="10"/>
@@ -21302,6 +21545,7 @@
         <v/>
       </c>
       <c r="J236" s="11"/>
+      <c r="K236" s="11"/>
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="10"/>
@@ -21323,6 +21567,7 @@
         <v/>
       </c>
       <c r="J237" s="11"/>
+      <c r="K237" s="11"/>
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="10"/>
@@ -21344,6 +21589,7 @@
         <v/>
       </c>
       <c r="J238" s="11"/>
+      <c r="K238" s="11"/>
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="10"/>
@@ -21365,6 +21611,7 @@
         <v/>
       </c>
       <c r="J239" s="11"/>
+      <c r="K239" s="11"/>
     </row>
     <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="10"/>
@@ -21386,6 +21633,7 @@
         <v/>
       </c>
       <c r="J240" s="11"/>
+      <c r="K240" s="11"/>
     </row>
     <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="10"/>
@@ -21407,6 +21655,7 @@
         <v/>
       </c>
       <c r="J241" s="11"/>
+      <c r="K241" s="11"/>
     </row>
     <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="10"/>
@@ -21428,6 +21677,7 @@
         <v/>
       </c>
       <c r="J242" s="11"/>
+      <c r="K242" s="11"/>
     </row>
     <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="10"/>
@@ -21449,6 +21699,7 @@
         <v/>
       </c>
       <c r="J243" s="11"/>
+      <c r="K243" s="11"/>
     </row>
     <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="10"/>
@@ -21470,6 +21721,7 @@
         <v/>
       </c>
       <c r="J244" s="11"/>
+      <c r="K244" s="11"/>
     </row>
     <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="10"/>
@@ -21491,6 +21743,7 @@
         <v/>
       </c>
       <c r="J245" s="11"/>
+      <c r="K245" s="11"/>
     </row>
     <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="10"/>
@@ -21512,6 +21765,7 @@
         <v/>
       </c>
       <c r="J246" s="11"/>
+      <c r="K246" s="11"/>
     </row>
     <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="10"/>
@@ -21533,6 +21787,7 @@
         <v/>
       </c>
       <c r="J247" s="11"/>
+      <c r="K247" s="11"/>
     </row>
     <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="10"/>
@@ -21554,6 +21809,7 @@
         <v/>
       </c>
       <c r="J248" s="11"/>
+      <c r="K248" s="11"/>
     </row>
     <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="10"/>
@@ -21575,6 +21831,7 @@
         <v/>
       </c>
       <c r="J249" s="11"/>
+      <c r="K249" s="11"/>
     </row>
     <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="10"/>
@@ -21596,6 +21853,7 @@
         <v/>
       </c>
       <c r="J250" s="11"/>
+      <c r="K250" s="11"/>
     </row>
     <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="10"/>
@@ -21617,6 +21875,7 @@
         <v/>
       </c>
       <c r="J251" s="11"/>
+      <c r="K251" s="11"/>
     </row>
     <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="10"/>
@@ -21638,6 +21897,7 @@
         <v/>
       </c>
       <c r="J252" s="11"/>
+      <c r="K252" s="11"/>
     </row>
     <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="10"/>
@@ -21659,6 +21919,7 @@
         <v/>
       </c>
       <c r="J253" s="11"/>
+      <c r="K253" s="11"/>
     </row>
     <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="10"/>
@@ -21680,6 +21941,7 @@
         <v/>
       </c>
       <c r="J254" s="11"/>
+      <c r="K254" s="11"/>
     </row>
     <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="10"/>
@@ -21701,6 +21963,7 @@
         <v/>
       </c>
       <c r="J255" s="11"/>
+      <c r="K255" s="11"/>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="10"/>
@@ -21722,6 +21985,7 @@
         <v/>
       </c>
       <c r="J256" s="11"/>
+      <c r="K256" s="11"/>
     </row>
     <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="10"/>
@@ -21743,6 +22007,7 @@
         <v/>
       </c>
       <c r="J257" s="11"/>
+      <c r="K257" s="11"/>
     </row>
     <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="10"/>
@@ -21764,6 +22029,7 @@
         <v/>
       </c>
       <c r="J258" s="11"/>
+      <c r="K258" s="11"/>
     </row>
     <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="10"/>
@@ -21785,6 +22051,7 @@
         <v/>
       </c>
       <c r="J259" s="11"/>
+      <c r="K259" s="11"/>
     </row>
     <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="10"/>
@@ -21806,6 +22073,7 @@
         <v/>
       </c>
       <c r="J260" s="11"/>
+      <c r="K260" s="11"/>
     </row>
     <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="10"/>
@@ -21827,6 +22095,7 @@
         <v/>
       </c>
       <c r="J261" s="11"/>
+      <c r="K261" s="11"/>
     </row>
     <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="10"/>
@@ -21848,6 +22117,7 @@
         <v/>
       </c>
       <c r="J262" s="11"/>
+      <c r="K262" s="11"/>
     </row>
     <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="10"/>
@@ -21869,6 +22139,7 @@
         <v/>
       </c>
       <c r="J263" s="11"/>
+      <c r="K263" s="11"/>
     </row>
     <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="10"/>
@@ -21890,6 +22161,7 @@
         <v/>
       </c>
       <c r="J264" s="11"/>
+      <c r="K264" s="11"/>
     </row>
     <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="10"/>
@@ -21911,6 +22183,7 @@
         <v/>
       </c>
       <c r="J265" s="11"/>
+      <c r="K265" s="11"/>
     </row>
     <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="10"/>
@@ -21932,6 +22205,7 @@
         <v/>
       </c>
       <c r="J266" s="11"/>
+      <c r="K266" s="11"/>
     </row>
     <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="10"/>
@@ -21953,6 +22227,7 @@
         <v/>
       </c>
       <c r="J267" s="11"/>
+      <c r="K267" s="11"/>
     </row>
     <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="10"/>
@@ -21974,6 +22249,7 @@
         <v/>
       </c>
       <c r="J268" s="11"/>
+      <c r="K268" s="11"/>
     </row>
     <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="10"/>
@@ -21995,6 +22271,7 @@
         <v/>
       </c>
       <c r="J269" s="11"/>
+      <c r="K269" s="11"/>
     </row>
     <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="10"/>
@@ -22016,6 +22293,7 @@
         <v/>
       </c>
       <c r="J270" s="11"/>
+      <c r="K270" s="11"/>
     </row>
     <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="10"/>
@@ -22037,6 +22315,7 @@
         <v/>
       </c>
       <c r="J271" s="11"/>
+      <c r="K271" s="11"/>
     </row>
     <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="10"/>
@@ -22058,6 +22337,7 @@
         <v/>
       </c>
       <c r="J272" s="11"/>
+      <c r="K272" s="11"/>
     </row>
     <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="10"/>
@@ -22079,6 +22359,7 @@
         <v/>
       </c>
       <c r="J273" s="11"/>
+      <c r="K273" s="11"/>
     </row>
     <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="10"/>
@@ -22100,6 +22381,7 @@
         <v/>
       </c>
       <c r="J274" s="11"/>
+      <c r="K274" s="11"/>
     </row>
     <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="10"/>
@@ -22121,6 +22403,7 @@
         <v/>
       </c>
       <c r="J275" s="11"/>
+      <c r="K275" s="11"/>
     </row>
     <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="10"/>
@@ -22142,6 +22425,7 @@
         <v/>
       </c>
       <c r="J276" s="11"/>
+      <c r="K276" s="11"/>
     </row>
     <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="10"/>
@@ -22163,6 +22447,7 @@
         <v/>
       </c>
       <c r="J277" s="11"/>
+      <c r="K277" s="11"/>
     </row>
     <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="10"/>
@@ -22184,6 +22469,7 @@
         <v/>
       </c>
       <c r="J278" s="11"/>
+      <c r="K278" s="11"/>
     </row>
     <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="10"/>
@@ -22205,6 +22491,7 @@
         <v/>
       </c>
       <c r="J279" s="11"/>
+      <c r="K279" s="11"/>
     </row>
     <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="10"/>
@@ -22226,6 +22513,7 @@
         <v/>
       </c>
       <c r="J280" s="11"/>
+      <c r="K280" s="11"/>
     </row>
     <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="10"/>
@@ -22247,6 +22535,7 @@
         <v/>
       </c>
       <c r="J281" s="11"/>
+      <c r="K281" s="11"/>
     </row>
     <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="10"/>
@@ -22268,6 +22557,7 @@
         <v/>
       </c>
       <c r="J282" s="11"/>
+      <c r="K282" s="11"/>
     </row>
     <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="10"/>
@@ -22289,6 +22579,7 @@
         <v/>
       </c>
       <c r="J283" s="11"/>
+      <c r="K283" s="11"/>
     </row>
     <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="10"/>
@@ -22310,6 +22601,7 @@
         <v/>
       </c>
       <c r="J284" s="11"/>
+      <c r="K284" s="11"/>
     </row>
     <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="10"/>
@@ -22331,6 +22623,7 @@
         <v/>
       </c>
       <c r="J285" s="11"/>
+      <c r="K285" s="11"/>
     </row>
     <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="10"/>
@@ -22352,6 +22645,7 @@
         <v/>
       </c>
       <c r="J286" s="11"/>
+      <c r="K286" s="11"/>
     </row>
     <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="10"/>
@@ -22373,6 +22667,7 @@
         <v/>
       </c>
       <c r="J287" s="11"/>
+      <c r="K287" s="11"/>
     </row>
     <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="10"/>
@@ -22394,6 +22689,7 @@
         <v/>
       </c>
       <c r="J288" s="11"/>
+      <c r="K288" s="11"/>
     </row>
     <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="10"/>
@@ -22415,6 +22711,7 @@
         <v/>
       </c>
       <c r="J289" s="11"/>
+      <c r="K289" s="11"/>
     </row>
     <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="10"/>
@@ -22436,6 +22733,7 @@
         <v/>
       </c>
       <c r="J290" s="11"/>
+      <c r="K290" s="11"/>
     </row>
     <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="10"/>
@@ -22457,6 +22755,7 @@
         <v/>
       </c>
       <c r="J291" s="11"/>
+      <c r="K291" s="11"/>
     </row>
     <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="10"/>
@@ -22478,6 +22777,7 @@
         <v/>
       </c>
       <c r="J292" s="11"/>
+      <c r="K292" s="11"/>
     </row>
     <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="10"/>
@@ -22499,6 +22799,7 @@
         <v/>
       </c>
       <c r="J293" s="11"/>
+      <c r="K293" s="11"/>
     </row>
     <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A294" s="10"/>
@@ -22520,6 +22821,7 @@
         <v/>
       </c>
       <c r="J294" s="11"/>
+      <c r="K294" s="11"/>
     </row>
     <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="10"/>
@@ -22541,6 +22843,7 @@
         <v/>
       </c>
       <c r="J295" s="11"/>
+      <c r="K295" s="11"/>
     </row>
     <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="10"/>
@@ -22562,6 +22865,7 @@
         <v/>
       </c>
       <c r="J296" s="11"/>
+      <c r="K296" s="11"/>
     </row>
     <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="10"/>
@@ -22583,6 +22887,7 @@
         <v/>
       </c>
       <c r="J297" s="11"/>
+      <c r="K297" s="11"/>
     </row>
     <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="10"/>
@@ -22604,6 +22909,7 @@
         <v/>
       </c>
       <c r="J298" s="11"/>
+      <c r="K298" s="11"/>
     </row>
     <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="10"/>
@@ -22625,6 +22931,7 @@
         <v/>
       </c>
       <c r="J299" s="11"/>
+      <c r="K299" s="11"/>
     </row>
     <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="10"/>
@@ -22646,6 +22953,7 @@
         <v/>
       </c>
       <c r="J300" s="11"/>
+      <c r="K300" s="11"/>
     </row>
     <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="10"/>
@@ -22667,14 +22975,21 @@
         <v/>
       </c>
       <c r="J301" s="11"/>
+      <c r="K301" s="11"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J301"/>
+  <autoFilter ref="A1:K301"/>
   <conditionalFormatting sqref="I2:I301">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>AND($I2&lt;&gt;"",$I2&lt;&gt;"OK")</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K301" type="list">
+      <formula1>"Téléphone,E-mail,Message,En boutique"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>